<commit_message>
Add transformers generation code (Gemma 12B, Phi-4, Ministral 3, BioMistral, PMC-LLaMA) and update settings table
</commit_message>
<xml_diff>
--- a/1_generation_code/model_settings/llm_generation_settings.xlsx
+++ b/1_generation_code/model_settings/llm_generation_settings.xlsx
@@ -2091,9 +2091,9 @@
           <t>General (open weights, local)</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>NOT RECORDED (slug 'gemma-4-12B-it')</t>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>google/gemma-4-12B-it</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2103,52 +2103,52 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>External local run (gemma12B)</t>
+          <t>Local transformers run on one NVIDIA RTX PRO 6000 Blackwell (96 GB); transformers 5.17.0, torch 2.10.0+cu128; chat template with separate system and user messages</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5 (seeds 1234-1238)</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Single sample, no selection</t>
-        </is>
-      </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>NOT RECORDED</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>NOT RECORDED</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t>NOT RECORDED</t>
-        </is>
-      </c>
-      <c r="L20" s="3" t="inlineStr">
-        <is>
-          <t>NOT RECORDED</t>
-        </is>
-      </c>
-      <c r="M20" s="3" t="inlineStr">
-        <is>
-          <t>NOT RECORDED</t>
-        </is>
-      </c>
-      <c r="N20" s="3" t="inlineStr">
-        <is>
-          <t>NOT RECORDED</t>
-        </is>
-      </c>
-      <c r="O20" s="3" t="inlineStr">
-        <is>
-          <t>NOT RECORDED</t>
+          <t>Medoid of the 5 answers: highest mean cosine similarity of all-MiniLM-L6-v2 embeddings (select_consistent.py). Only the selected answer is stored in the repository</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>top_k 64 (the checkpoint's own generation_config.json values)</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>1,024 (cap = effective context - prompt length - 16, not reached)</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Not set</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>bfloat16</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>1234-1238</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>gemma12B/*.json (keys: model, answer only); convert_gemma12b_results.py</t>
+          <t>LLM_codes_RTX6000station README.md, parameters.csv and scripts; gemma12B/scripts/*</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2188,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>External local run (phi4_14B_results; Hugging Face-style arguments)</t>
+          <t>Local transformers run on one NVIDIA RTX PRO 6000 Blackwell (96 GB); chat template with separate system and user messages; transformers version not recorded</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>none recorded</t>
+          <t>top_k not set</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2226,9 +2226,9 @@
           <t>No thinking mode</t>
         </is>
       </c>
-      <c r="N21" s="3" t="inlineStr">
-        <is>
-          <t>NOT RECORDED</t>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>bfloat16</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>phi4_14B_results/*.json -&gt; generation_settings; convert_phi4_ministral_results.py</t>
+          <t>LLM_codes_RTX6000station README.md, parameters.csv and scripts; phi4_14B/run_inference.py and the saved result files</t>
         </is>
       </c>
     </row>
@@ -2253,7 +2253,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Ministral 3 14B (Reasoning)</t>
+          <t>Ministral 3 14B</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>External local run (ministral3_14B_results)</t>
+          <t>External local run. The saved answers that were evaluated come from unsloth/Ministral-3-14B-Reasoning-2512-bnb-4bit; the script supplied in local_models_transformers/ministral3_14B runs mistralai/Ministral-3-14B-Base-2512 in bf16 (temperature 1.0, top_p 0.9, repetition_penalty 1.05, no_repeat_ngram_size 3, max_new_tokens 1,536, seed 1234, plain concatenation of system and user text) and did not produce the evaluated answers</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>ministral3_14B_results/*.json -&gt; generation_settings; convert_phi4_ministral_results.py</t>
+          <t>ministral3_14B_results/*.json -&gt; generation_settings; convert_phi4_ministral_results.py; LLM_codes_RTX6000station README.md, parameters.csv and scripts; ministral3_14B/run_inference.py</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>External local run (bioLLM/biomistral)</t>
+          <t>Local transformers run on one NVIDIA RTX PRO 6000 Blackwell (96 GB); transformers 5.2.0, torch 2.10.0+cu128; chat template, system text folded into the user turn, response-format directive appended to the prompt at run time</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -2396,14 +2396,14 @@
           <t>None (base biomedical model)</t>
         </is>
       </c>
-      <c r="N23" s="3" t="inlineStr">
-        <is>
-          <t>NOT RECORDED</t>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>bfloat16</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Different seed per run, stored in the source jsonl</t>
+          <t>1234-1238 (one per run)</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -2413,7 +2413,7 @@
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>bioLLM/biomistral/*.jsonl -&gt; generation_settings; convert_biollm_results.py</t>
+          <t>LLM_codes_RTX6000station README.md, parameters.csv and scripts; bioLLM/scripts/*; bioLLM/biomistral/*.jsonl</t>
         </is>
       </c>
     </row>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>External local run (bioLLM/pmc_llama)</t>
+          <t>Local transformers run on one NVIDIA RTX PRO 6000 Blackwell (96 GB); transformers 5.2.0, torch 2.10.0+cu128; plain concatenation of system and user text (no chat template), completion directive ending 'PRIMARY ZONE:', slow LlamaTokenizer, RoPE linear scaling x2 (4,096-token context)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2481,14 +2481,14 @@
           <t>None (base biomedical model)</t>
         </is>
       </c>
-      <c r="N24" s="3" t="inlineStr">
-        <is>
-          <t>NOT RECORDED</t>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>float32 (native)</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Different seed per run, stored in the source jsonl</t>
+          <t>1234-1238 (one per run)</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -2498,7 +2498,7 @@
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>bioLLM/pmc_llama/*.jsonl -&gt; generation_settings; convert_biollm_results.py</t>
+          <t>LLM_codes_RTX6000station README.md, parameters.csv and scripts; bioLLM/scripts/*; bioLLM/pmc_llama/*.jsonl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename the 9B Qwen run to Qwen3.5-9B (folders, files, tables, figures); regenerate figures from the renamed data
</commit_message>
<xml_diff>
--- a/1_generation_code/model_settings/llm_generation_settings.xlsx
+++ b/1_generation_code/model_settings/llm_generation_settings.xlsx
@@ -1998,7 +1998,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Qwen 9B (thinking, temp 1) [slug: Qwen3.8-9B-think-temp1]</t>
+          <t>Qwen3.5-9B (thinking, temp 1)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Qwen/Qwen3.5-9B per configs/case_studies_think_t1.json (the answer folder is named Qwen3.8-9B-think-temp1)</t>
+          <t>Qwen/Qwen3.5-9B (configs/case_studies_think_t1.json)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Ministral 3 14B: replace the Base-2512 scripts with the Reasoning-2512 scripts that generated the evaluated answers
run_inference_reasoning.py + export_clean_reasoning_results.py (unsloth/Ministral-3-14B-Reasoning-2512-bnb-4bit, temperature 0.3, top_p 0.9,
max_new_tokens 4096, seed 1234). README, parameters.csv and llm_generation_settings.xlsx updated; the Base-2512 trial is noted as not used for any evaluation.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/1_generation_code/model_settings/llm_generation_settings.xlsx
+++ b/1_generation_code/model_settings/llm_generation_settings.xlsx
@@ -2273,7 +2273,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>External local run. The saved answers that were evaluated come from unsloth/Ministral-3-14B-Reasoning-2512-bnb-4bit; the script supplied in local_models_transformers/ministral3_14B runs mistralai/Ministral-3-14B-Base-2512 in bf16 (temperature 1.0, top_p 0.9, repetition_penalty 1.05, no_repeat_ngram_size 3, max_new_tokens 1,536, seed 1234, plain concatenation of system and user text) and did not produce the evaluated answers</t>
+          <t>External local run with ministral3_14B/run_inference_reasoning.py (Hugging Face transformers, Mistral3ForConditionalGeneration, chat template with separate system and user messages, [THINK] block split from the answer), cleaned by export_clean_reasoning_results.py. The saved results_clean files are the evaluated answers. An earlier trial with Ministral-3-14B-Base-2512 was not used for any evaluation.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>ministral3_14B_results/*.json -&gt; generation_settings; convert_phi4_ministral_results.py; LLM_codes_RTX6000station README.md, parameters.csv and scripts; ministral3_14B/run_inference.py</t>
+          <t>ministral3_14B/run_inference_reasoning.py and export_clean_reasoning_results.py; ministral3_14B_reasoning_results_clean/*.json -&gt; generation_settings; convert_phi4_ministral_results.py</t>
         </is>
       </c>
     </row>

</xml_diff>